<commit_message>
Build #3 - FAILURE
</commit_message>
<xml_diff>
--- a/test-reports/Board_Test_Report.xlsx
+++ b/test-reports/Board_Test_Report.xlsx
@@ -513,7 +513,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>#29</t>
+          <t>#3</t>
         </is>
       </c>
     </row>
@@ -525,7 +525,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Tuesday 30 June 2026 04:38:31 PM IST</t>
+          <t>Wednesday 01 July 2026 10:58:46 AM IST</t>
         </is>
       </c>
     </row>
@@ -561,7 +561,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>local-ssh-agent</t>
+          <t>ssh-agent-key</t>
         </is>
       </c>
     </row>
@@ -602,16 +602,17 @@
     <row r="10" ht="345.5" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>+ ping -c 3 192.168.11.173
+          <t>+ echo === Ping Test ===
+=== Ping Test ===
++ ping -c 3 192.168.11.173
 PING 192.168.11.173 (192.168.11.173) 56(84) bytes of data.
 --- 192.168.11.173 ping statistics ---
-3 packets transmitted, 0 received, 100% packet loss, time 2079ms</t>
+3 packets transmitted, 0 received, 100% packet loss, time 2052ms</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>+ ssh -o StrictHostKeyChecking=no root@192.168.11.173 echo ✅ SSH Connected! &amp;&amp; hostname &amp;&amp; uptime
-Terminated</t>
+          <t>(no output captured)</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">

</xml_diff>